<commit_message>
Snabb produktinmatning + Faktor-fält för enkla produkter, uppdaterade Excel-mallar
Lägger till ett rutnätsbaserat snabbinmatningsläge för att skapa flera enkla
produkter i rad (samma UX-mönster som bänkskivor), samma "Faktor"-fält som
redan finns för variantprodukter (inköpspris x faktor x moms -> försäljningspris),
och ordnar om prisfälten i produktformuläret till inköpspris - faktor -
försäljningspris - montage - montörens del. Döper också om "Försäljningspris
Montage" till "Montagekostnad". Excel-mallen för enkla produkter är uppdaterad
med samma fältordning och en Faktor-kolumn, och importlogiken i products.html
är uppdaterad för att matcha de nya kolumnrubrikerna.

Kräver att migrations/2026-07-24_product_markup_factor.sql körs mot databasen.
</commit_message>
<xml_diff>
--- a/public/mallar/Mall_Enkla_produkter.xlsx
+++ b/public/mallar/Mall_Enkla_produkter.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -577,33 +577,47 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Försäljningspris Montage / Montörens del - lämna som 0 om produkten inte har montagekostnad.</t>
+          <t>Faktor - valfri hjälpkolumn (samma som i systemets snabbinmatning). Fylls INTE i något prisfält automatiskt vid</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  import från Excel (till skillnad från i själva systemet) - du sätter ändå försäljningspriset manuellt här.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Montagekostnad / Montörens del - lämna som 0 om produkten inte har montagekostnad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>Stommens mått - fyll bara i för skåpstommar som ska ha automatisk lucka/lådfrontberäkning (annars lämna tomt/0).</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Fälten som INTE finns i denna mall** (leverantör, dörrmodell-koppling, tillbehörsgrupp, bilder) sätts enklast manuellt</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>på produkten efter import, om det behövs - annars fungerar produkten fint utan dem.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Exempelraderna (kursiv grå text) visar formatet för både styckpris och per m²-prissättning - radera dem innan import.</t>
         </is>
@@ -620,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -629,15 +643,16 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -673,45 +688,50 @@
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
+          <t>Inköpspris (kr)</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Faktor</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
           <t>Försäljningspris Material (kr, inkl moms)</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>Pris per m² (kr, inkl moms)</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>Minsta debiterbar yta (m²)</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
-        <is>
-          <t>Försäljningspris Montage (kr, inkl moms)</t>
-        </is>
-      </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>Montagekostnad (kr, inkl moms)</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>Montörens del av montage (kr)</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
-        <is>
-          <t>Inköpspris (kr)</t>
-        </is>
-      </c>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="N1" s="5" t="inlineStr">
         <is>
           <t>Stommens höjd (mm)</t>
         </is>
       </c>
-      <c r="N1" s="5" t="inlineStr">
+      <c r="O1" s="5" t="inlineStr">
         <is>
           <t>Stommens bredd (mm)</t>
         </is>
       </c>
-      <c r="O1" s="5" t="inlineStr">
+      <c r="P1" s="5" t="inlineStr">
         <is>
           <t>Stommens djup (mm)</t>
         </is>
@@ -749,22 +769,23 @@
         </is>
       </c>
       <c r="G2" s="6" t="n">
+        <v>95</v>
+      </c>
+      <c r="H2" s="6" t="n"/>
+      <c r="I2" s="6" t="n">
         <v>189</v>
       </c>
-      <c r="H2" s="6" t="n"/>
-      <c r="I2" s="6" t="n"/>
-      <c r="J2" s="6" t="n">
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="6" t="n"/>
+      <c r="L2" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="K2" s="6" t="n">
+      <c r="M2" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="L2" s="6" t="n">
-        <v>95</v>
-      </c>
-      <c r="M2" s="6" t="n"/>
       <c r="N2" s="6" t="n"/>
       <c r="O2" s="6" t="n"/>
+      <c r="P2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -793,25 +814,26 @@
           <t>Per m²</t>
         </is>
       </c>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n">
+      <c r="G3" s="6" t="n">
+        <v>620</v>
+      </c>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="6" t="n">
         <v>1450</v>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="K3" s="6" t="n">
         <v>0.5</v>
       </c>
-      <c r="J3" s="6" t="n">
+      <c r="L3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="K3" s="6" t="n">
+      <c r="M3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="L3" s="6" t="n">
-        <v>620</v>
-      </c>
-      <c r="M3" s="6" t="n"/>
       <c r="N3" s="6" t="n"/>
       <c r="O3" s="6" t="n"/>
+      <c r="P3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n"/>
@@ -829,6 +851,7 @@
       <c r="M4" s="7" t="n"/>
       <c r="N4" s="7" t="n"/>
       <c r="O4" s="7" t="n"/>
+      <c r="P4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n"/>
@@ -846,6 +869,7 @@
       <c r="M5" s="7" t="n"/>
       <c r="N5" s="7" t="n"/>
       <c r="O5" s="7" t="n"/>
+      <c r="P5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n"/>
@@ -863,6 +887,7 @@
       <c r="M6" s="7" t="n"/>
       <c r="N6" s="7" t="n"/>
       <c r="O6" s="7" t="n"/>
+      <c r="P6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n"/>
@@ -880,6 +905,7 @@
       <c r="M7" s="7" t="n"/>
       <c r="N7" s="7" t="n"/>
       <c r="O7" s="7" t="n"/>
+      <c r="P7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n"/>
@@ -897,6 +923,7 @@
       <c r="M8" s="7" t="n"/>
       <c r="N8" s="7" t="n"/>
       <c r="O8" s="7" t="n"/>
+      <c r="P8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n"/>
@@ -914,6 +941,7 @@
       <c r="M9" s="7" t="n"/>
       <c r="N9" s="7" t="n"/>
       <c r="O9" s="7" t="n"/>
+      <c r="P9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n"/>
@@ -931,6 +959,7 @@
       <c r="M10" s="7" t="n"/>
       <c r="N10" s="7" t="n"/>
       <c r="O10" s="7" t="n"/>
+      <c r="P10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -948,6 +977,7 @@
       <c r="M11" s="7" t="n"/>
       <c r="N11" s="7" t="n"/>
       <c r="O11" s="7" t="n"/>
+      <c r="P11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n"/>
@@ -965,6 +995,7 @@
       <c r="M12" s="7" t="n"/>
       <c r="N12" s="7" t="n"/>
       <c r="O12" s="7" t="n"/>
+      <c r="P12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n"/>
@@ -982,6 +1013,7 @@
       <c r="M13" s="7" t="n"/>
       <c r="N13" s="7" t="n"/>
       <c r="O13" s="7" t="n"/>
+      <c r="P13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -999,6 +1031,7 @@
       <c r="M14" s="7" t="n"/>
       <c r="N14" s="7" t="n"/>
       <c r="O14" s="7" t="n"/>
+      <c r="P14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>
@@ -1016,6 +1049,7 @@
       <c r="M15" s="7" t="n"/>
       <c r="N15" s="7" t="n"/>
       <c r="O15" s="7" t="n"/>
+      <c r="P15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n"/>
@@ -1033,6 +1067,7 @@
       <c r="M16" s="7" t="n"/>
       <c r="N16" s="7" t="n"/>
       <c r="O16" s="7" t="n"/>
+      <c r="P16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n"/>
@@ -1050,6 +1085,7 @@
       <c r="M17" s="7" t="n"/>
       <c r="N17" s="7" t="n"/>
       <c r="O17" s="7" t="n"/>
+      <c r="P17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n"/>
@@ -1067,6 +1103,7 @@
       <c r="M18" s="7" t="n"/>
       <c r="N18" s="7" t="n"/>
       <c r="O18" s="7" t="n"/>
+      <c r="P18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n"/>
@@ -1084,6 +1121,7 @@
       <c r="M19" s="7" t="n"/>
       <c r="N19" s="7" t="n"/>
       <c r="O19" s="7" t="n"/>
+      <c r="P19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n"/>
@@ -1101,6 +1139,7 @@
       <c r="M20" s="7" t="n"/>
       <c r="N20" s="7" t="n"/>
       <c r="O20" s="7" t="n"/>
+      <c r="P20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n"/>
@@ -1118,6 +1157,7 @@
       <c r="M21" s="7" t="n"/>
       <c r="N21" s="7" t="n"/>
       <c r="O21" s="7" t="n"/>
+      <c r="P21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n"/>
@@ -1135,6 +1175,7 @@
       <c r="M22" s="7" t="n"/>
       <c r="N22" s="7" t="n"/>
       <c r="O22" s="7" t="n"/>
+      <c r="P22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n"/>
@@ -1152,6 +1193,7 @@
       <c r="M23" s="7" t="n"/>
       <c r="N23" s="7" t="n"/>
       <c r="O23" s="7" t="n"/>
+      <c r="P23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n"/>
@@ -1169,6 +1211,7 @@
       <c r="M24" s="7" t="n"/>
       <c r="N24" s="7" t="n"/>
       <c r="O24" s="7" t="n"/>
+      <c r="P24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
@@ -1186,6 +1229,7 @@
       <c r="M25" s="7" t="n"/>
       <c r="N25" s="7" t="n"/>
       <c r="O25" s="7" t="n"/>
+      <c r="P25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n"/>
@@ -1203,6 +1247,7 @@
       <c r="M26" s="7" t="n"/>
       <c r="N26" s="7" t="n"/>
       <c r="O26" s="7" t="n"/>
+      <c r="P26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n"/>
@@ -1220,6 +1265,7 @@
       <c r="M27" s="7" t="n"/>
       <c r="N27" s="7" t="n"/>
       <c r="O27" s="7" t="n"/>
+      <c r="P27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n"/>
@@ -1237,6 +1283,7 @@
       <c r="M28" s="7" t="n"/>
       <c r="N28" s="7" t="n"/>
       <c r="O28" s="7" t="n"/>
+      <c r="P28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n"/>
@@ -1254,6 +1301,7 @@
       <c r="M29" s="7" t="n"/>
       <c r="N29" s="7" t="n"/>
       <c r="O29" s="7" t="n"/>
+      <c r="P29" s="7" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>